<commit_message>
add pile support for OMS method in LEM analysis
Parse piles sheet from Excel input (fileio.py), assign pile forces to
slices via geometric intersection (slice.py), add H·sin(α−θp) to N'
and pile resisting moment to OMS denominator (solve.py), and visualize
pile lines with intersection markers (plot.py).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_piles.xlsx
+++ b/docs/lem/files/xslope_piles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D7A10D-180F-6940-9091-BE39947CA342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D00CFB-5529-BF47-BD9D-90384999F2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6340" yWindow="3000" windowWidth="27840" windowHeight="20620" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="3880" yWindow="5600" windowWidth="33620" windowHeight="20620" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="179">
   <si>
     <t>X</t>
   </si>
@@ -724,6 +724,9 @@
   </si>
   <si>
     <t>soil</t>
+  </si>
+  <si>
+    <t>pile</t>
   </si>
 </sst>
 </file>
@@ -1165,19 +1168,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1208,21 +1211,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill>
@@ -7815,6 +7804,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -7824,6 +7819,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-10</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -10782,11 +10783,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="47" t="s">
+      <c r="B7" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -11846,12 +11847,24 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="B3" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C3" s="3">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3">
+        <v>-10</v>
+      </c>
+      <c r="G3" s="3">
+        <v>5000</v>
+      </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -13081,36 +13094,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="48"/>
-      <c r="J7" s="48"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="48" t="s">
+      <c r="L7" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="48"/>
-      <c r="N7" s="48"/>
-      <c r="O7" s="48"/>
-      <c r="P7" s="48"/>
-      <c r="Q7" s="48"/>
-      <c r="R7" s="48" t="s">
+      <c r="M7" s="47"/>
+      <c r="N7" s="47"/>
+      <c r="O7" s="47"/>
+      <c r="P7" s="47"/>
+      <c r="Q7" s="47"/>
+      <c r="R7" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="S7" s="48"/>
-      <c r="T7" s="48"/>
-      <c r="U7" s="48"/>
-      <c r="V7" s="48"/>
-      <c r="W7" s="48" t="s">
+      <c r="S7" s="47"/>
+      <c r="T7" s="47"/>
+      <c r="U7" s="47"/>
+      <c r="V7" s="47"/>
+      <c r="W7" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="X7" s="48"/>
+      <c r="X7" s="47"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -13898,38 +13911,33 @@
     <mergeCell ref="W7:X7"/>
     <mergeCell ref="R7:V7"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F50">
-    <cfRule type="expression" dxfId="10" priority="4">
-      <formula>$D10="cp"</formula>
+  <conditionalFormatting sqref="F9:F50">
+    <cfRule type="expression" dxfId="8" priority="1">
+      <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:H50">
-    <cfRule type="expression" dxfId="9" priority="3">
+    <cfRule type="expression" dxfId="7" priority="3">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:J50">
-    <cfRule type="expression" dxfId="8" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N9:N50">
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:O50">
-    <cfRule type="expression" dxfId="6" priority="14">
+    <cfRule type="expression" dxfId="4" priority="14">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9:Q50">
-    <cfRule type="expression" dxfId="5" priority="9">
-      <formula>$D9="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F9">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="3" priority="9">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13983,74 +13991,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="D4" s="51" t="s">
+      <c r="B4" s="49"/>
+      <c r="D4" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="51"/>
-      <c r="G4" s="51" t="s">
+      <c r="E4" s="49"/>
+      <c r="G4" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="51"/>
-      <c r="J4" s="51" t="s">
+      <c r="H4" s="49"/>
+      <c r="J4" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="51"/>
-      <c r="M4" s="51" t="s">
+      <c r="K4" s="49"/>
+      <c r="M4" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="51"/>
-      <c r="P4" s="51" t="s">
+      <c r="N4" s="49"/>
+      <c r="P4" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="51"/>
+      <c r="Q4" s="49"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="51" t="s">
+      <c r="S4" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="51"/>
+      <c r="T4" s="49"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="51" t="s">
+      <c r="V4" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="51"/>
+      <c r="W4" s="49"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="51" t="s">
+      <c r="Y4" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="51"/>
+      <c r="Z4" s="49"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="51" t="s">
+      <c r="AB4" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="51"/>
-      <c r="AE4" s="51" t="s">
+      <c r="AC4" s="49"/>
+      <c r="AE4" s="49" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="51"/>
+      <c r="AF4" s="49"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AH4" s="49" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="51"/>
+      <c r="AI4" s="49"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="51" t="s">
+      <c r="AK4" s="49" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="51"/>
+      <c r="AL4" s="49"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="51" t="s">
+      <c r="AN4" s="49" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="51"/>
+      <c r="AO4" s="49"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="51" t="s">
+      <c r="AQ4" s="49" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="51"/>
+      <c r="AR4" s="49"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -14153,89 +14161,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="49" t="str">
+      <c r="A6" s="50" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>soil</v>
       </c>
-      <c r="B6" s="50"/>
-      <c r="D6" s="49" t="str">
+      <c r="B6" s="51"/>
+      <c r="D6" s="50" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="50"/>
-      <c r="G6" s="49" t="str">
+      <c r="E6" s="51"/>
+      <c r="G6" s="50" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="50"/>
-      <c r="J6" s="49" t="str">
+      <c r="H6" s="51"/>
+      <c r="J6" s="50" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="50"/>
-      <c r="M6" s="49" t="str">
+      <c r="K6" s="51"/>
+      <c r="M6" s="50" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="50"/>
-      <c r="P6" s="49" t="str">
+      <c r="N6" s="51"/>
+      <c r="P6" s="50" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="50"/>
+      <c r="Q6" s="51"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="49" t="str">
+      <c r="S6" s="50" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="50"/>
+      <c r="T6" s="51"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="49" t="str">
+      <c r="V6" s="50" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="50"/>
+      <c r="W6" s="51"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="49" t="str">
+      <c r="Y6" s="50" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="50"/>
+      <c r="Z6" s="51"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="49" t="str">
+      <c r="AB6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="50"/>
-      <c r="AE6" s="49" t="str">
+      <c r="AC6" s="51"/>
+      <c r="AE6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="50"/>
+      <c r="AF6" s="51"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="49" t="str">
+      <c r="AH6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="50"/>
+      <c r="AI6" s="51"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="49" t="str">
+      <c r="AK6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="50"/>
+      <c r="AL6" s="51"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="49" t="str">
+      <c r="AN6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="50"/>
+      <c r="AO6" s="51"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="49" t="str">
+      <c r="AQ6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="50"/>
+      <c r="AR6" s="51"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -15155,36 +15163,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15222,74 +15230,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="D4" s="51" t="s">
+      <c r="B4" s="49"/>
+      <c r="D4" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="51"/>
-      <c r="G4" s="51" t="s">
+      <c r="E4" s="49"/>
+      <c r="G4" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="51"/>
-      <c r="J4" s="51" t="s">
+      <c r="H4" s="49"/>
+      <c r="J4" s="49" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="51"/>
-      <c r="M4" s="51" t="s">
+      <c r="K4" s="49"/>
+      <c r="M4" s="49" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="51"/>
-      <c r="P4" s="51" t="s">
+      <c r="N4" s="49"/>
+      <c r="P4" s="49" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="51"/>
+      <c r="Q4" s="49"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="51" t="s">
+      <c r="S4" s="49" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="51"/>
+      <c r="T4" s="49"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="51" t="s">
+      <c r="V4" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="51"/>
+      <c r="W4" s="49"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="51" t="s">
+      <c r="Y4" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="51"/>
+      <c r="Z4" s="49"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="51" t="s">
+      <c r="AB4" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="51"/>
-      <c r="AE4" s="51" t="s">
+      <c r="AC4" s="49"/>
+      <c r="AE4" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="51"/>
+      <c r="AF4" s="49"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AH4" s="49" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="51"/>
+      <c r="AI4" s="49"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="51" t="s">
+      <c r="AK4" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="51"/>
+      <c r="AL4" s="49"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="51" t="s">
+      <c r="AN4" s="49" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="51"/>
+      <c r="AO4" s="49"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="51" t="s">
+      <c r="AQ4" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="51"/>
+      <c r="AR4" s="49"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -16378,12 +16386,14 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -16400,14 +16410,12 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16773,24 +16781,19 @@
       <c r="N16" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E4:E42">
-    <cfRule type="expression" dxfId="4" priority="4">
-      <formula>OR($D4="Intercept", $D4="Radius")</formula>
+  <conditionalFormatting sqref="E3:E42">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>

<commit_message>
add Ito & Matsui auto-computation of pile force H
New module ito_matsui.py implements the Ito & Matsui (1975) closed-form
method for computing lateral force on passive piles. When H is left blank
in the piles sheet but D and S are provided, H is auto-computed at slice
generation time for each trial failure surface. The computed H is printed
after the search converges.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_piles.xlsx
+++ b/docs/lem/files/xslope_piles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D00CFB-5529-BF47-BD9D-90384999F2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B0BEC2-B169-4F40-A0DC-06CF86F0024A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3880" yWindow="5600" windowWidth="33620" windowHeight="20620" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="24840" yWindow="5860" windowWidth="37700" windowHeight="20620" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -10123,7 +10123,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>426357</xdr:colOff>
+      <xdr:colOff>27214</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>54428</xdr:rowOff>
     </xdr:to>
@@ -10141,7 +10141,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10885714" y="498930"/>
-          <a:ext cx="4826000" cy="2748641"/>
+          <a:ext cx="4426857" cy="2748641"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -11862,12 +11862,14 @@
       <c r="F3" s="3">
         <v>-10</v>
       </c>
-      <c r="G3" s="3">
-        <v>5000</v>
-      </c>
+      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="I3" s="3">
+        <v>3</v>
+      </c>
+      <c r="J3" s="3">
+        <v>10</v>
+      </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>

</xml_diff>

<commit_message>
add pile sample problem and Ito & Matsui summary output
Add sample 10 (pile-stabilized slope) to LEM samples with input,
no-pile, and with-pile solution images. Print full Ito & Matsui
summary table (D, S, D1, depth, A1, A2, F_pile, H) after search.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_piles.xlsx
+++ b/docs/lem/files/xslope_piles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B0BEC2-B169-4F40-A0DC-06CF86F0024A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4165D0BA-76A5-DE41-B428-E4428D9DDA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24840" yWindow="5860" windowWidth="37700" windowHeight="20620" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="31620" yWindow="5880" windowWidth="37700" windowHeight="20620" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1168,19 +1168,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1364,7 +1364,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>90</c:v>
@@ -7820,7 +7820,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>5</c:v>
+                  <c:v>6.67</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-10</c:v>
@@ -10783,11 +10783,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -11854,7 +11854,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="3">
-        <v>5</v>
+        <v>6.67</v>
       </c>
       <c r="E3" s="3">
         <v>10</v>
@@ -11865,10 +11865,10 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J3" s="3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
@@ -13096,36 +13096,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="47"/>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="47"/>
-      <c r="I7" s="47"/>
-      <c r="J7" s="47"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="47" t="s">
+      <c r="L7" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="47"/>
-      <c r="N7" s="47"/>
-      <c r="O7" s="47"/>
-      <c r="P7" s="47"/>
-      <c r="Q7" s="47"/>
-      <c r="R7" s="47" t="s">
+      <c r="M7" s="48"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="48"/>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="48"/>
+      <c r="R7" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S7" s="47"/>
-      <c r="T7" s="47"/>
-      <c r="U7" s="47"/>
-      <c r="V7" s="47"/>
-      <c r="W7" s="47" t="s">
+      <c r="S7" s="48"/>
+      <c r="T7" s="48"/>
+      <c r="U7" s="48"/>
+      <c r="V7" s="48"/>
+      <c r="W7" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="X7" s="47"/>
+      <c r="X7" s="48"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -13209,16 +13209,16 @@
         <v>177</v>
       </c>
       <c r="C9" s="3">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E9" s="3">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="F9" s="3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -13993,74 +13993,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="D4" s="49" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="G4" s="49" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="49"/>
-      <c r="J4" s="49" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="49"/>
-      <c r="M4" s="49" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="49"/>
-      <c r="P4" s="49" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="49"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="49" t="s">
+      <c r="S4" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="49"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="49" t="s">
+      <c r="V4" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="49"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="49" t="s">
+      <c r="Y4" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="49"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="49" t="s">
+      <c r="AB4" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="49"/>
-      <c r="AE4" s="49" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="49"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="49" t="s">
+      <c r="AH4" s="51" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="49"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="49" t="s">
+      <c r="AK4" s="51" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="49"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="49" t="s">
+      <c r="AN4" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="49"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="49" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="49"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -14163,89 +14163,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="str">
+      <c r="A6" s="49" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>soil</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="D6" s="50" t="str">
+      <c r="B6" s="50"/>
+      <c r="D6" s="49" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="51"/>
-      <c r="G6" s="50" t="str">
+      <c r="E6" s="50"/>
+      <c r="G6" s="49" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="51"/>
-      <c r="J6" s="50" t="str">
+      <c r="H6" s="50"/>
+      <c r="J6" s="49" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="51"/>
-      <c r="M6" s="50" t="str">
+      <c r="K6" s="50"/>
+      <c r="M6" s="49" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="51"/>
-      <c r="P6" s="50" t="str">
+      <c r="N6" s="50"/>
+      <c r="P6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="51"/>
+      <c r="Q6" s="50"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="50" t="str">
+      <c r="S6" s="49" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="51"/>
+      <c r="T6" s="50"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="50" t="str">
+      <c r="V6" s="49" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="51"/>
+      <c r="W6" s="50"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="50" t="str">
+      <c r="Y6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="51"/>
+      <c r="Z6" s="50"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="50" t="str">
+      <c r="AB6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="51"/>
-      <c r="AE6" s="50" t="str">
+      <c r="AC6" s="50"/>
+      <c r="AE6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="51"/>
+      <c r="AF6" s="50"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="50" t="str">
+      <c r="AH6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="51"/>
+      <c r="AI6" s="50"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="50" t="str">
+      <c r="AK6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="51"/>
+      <c r="AL6" s="50"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="50" t="str">
+      <c r="AN6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="51"/>
+      <c r="AO6" s="50"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="50" t="str">
+      <c r="AQ6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="51"/>
+      <c r="AR6" s="50"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -14437,7 +14437,7 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B10" s="3">
         <v>20</v>
@@ -15165,36 +15165,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15232,74 +15232,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="D4" s="49" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="G4" s="49" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="49"/>
-      <c r="J4" s="49" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="49"/>
-      <c r="M4" s="49" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="49"/>
-      <c r="P4" s="49" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="49"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="49" t="s">
+      <c r="S4" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="49"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="49" t="s">
+      <c r="V4" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="49"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="49" t="s">
+      <c r="Y4" s="51" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="49"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="49" t="s">
+      <c r="AB4" s="51" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="49"/>
-      <c r="AE4" s="49" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="49"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="49" t="s">
+      <c r="AH4" s="51" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="49"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="49" t="s">
+      <c r="AK4" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="49"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="49" t="s">
+      <c r="AN4" s="51" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="49"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="49" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="49"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -16388,14 +16388,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -16412,12 +16410,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs+data(tutorials): the pile rows carry unique labels, and the theta-p clause reads plainly
Owner flag on the editor screenshot: both rows were labeled 'pile'. The
sample file now names them 'lower row' and 'upper row' (label cells edited
by XML surgery — the file is hand-maintained, no builder — leaving the
rich-text headers untouched; loader reads the new labels and the critical
FS holds at 1.842). The tutorial's sheet and report tables match, and the
six LEM-12 Studio captures regenerate. The table-view sentence now says
why there is no theta-p column instead of compressing it into a clause.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_piles.xlsx
+++ b/docs/lem/files/xslope_piles.xlsx
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>pile</t>
+          <t>lower row</t>
         </is>
       </c>
       <c r="C3" s="3">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>pile</t>
+          <t>upper row</t>
         </is>
       </c>
       <c r="C4" s="3">

</xml_diff>

<commit_message>
data+docs(piles): saved files spell Appl out — a default nobody can see is a trap
Owner ruling: the writer now writes Active/Passive explicitly (as it
already did Fixity's free), so saved and auto-upgraded files self-document;
a blank cell still loads as active for old and hand-built files, and the
template docs say both halves. The sample re-saved through the round trip
(categories identical, FS 1.842), its rendered sheet shows Active, and
LEM-12's table matches the editor screenshot instead of needing a sentence
to explain why they disagreed. Reinforce-sheet Dir/Appl held for a separate
look per the owner (Type-preset formulas interact).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_piles.xlsx
+++ b/docs/lem/files/xslope_piles.xlsx
@@ -3991,7 +3991,11 @@
         <v>-10.0</v>
       </c>
       <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="I3" s="3">
         <v>2.0</v>
       </c>
@@ -4043,7 +4047,11 @@
         <v>-10.0</v>
       </c>
       <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="I4" s="3">
         <v>2.0</v>
       </c>

</xml_diff>

<commit_message>
data(piles): the pile row model declares t_cut = 0
The model behind LEM sample problem 10, LEM-12 and FEM-3's first half left the
tensile cutoff blank on its one Mohr-Coulomb row, so Run FEM raised the
unbounded-tension warning and the clay was free to carry tension up to
c/tan(phi) = 549.5 psf under the pile rows. It now declares t_cut = 0.

Written through xslope.fileio.write_cells_to_xlsx; the cell-level diff is
mat!L11 and nothing else, and load_slope_data reads 0.0 back. The limit
equilibrium answers on the file are untouched -- t_cut is read by xslope/fem.py
alone -- so sample problem 10's Spencer lock and LEM-12's numbers stand. The
finite element answers on FEM-3 move and are re-measured on that page.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_piles.xlsx
+++ b/docs/lem/files/xslope_piles.xlsx
@@ -6612,7 +6612,9 @@
       <c r="K11" s="3">
         <v>0.0</v>
       </c>
-      <c r="L11" s="3"/>
+      <c r="L11" s="3">
+        <v>0</v>
+      </c>
       <c r="M11" s="3">
         <v>2000000.0</v>
       </c>

</xml_diff>